<commit_message>
LMDI: Merge pull request #62 from folkehelseinstituttet/fix/presisering-npr-episode-identifier
Presiser dokumentasjon for NPR episodeidentifikator bd1d3b6e2e552e20cf9b98e8205a970bf6b66351
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-encounter.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-encounter.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-13T18:31:12+00:00</t>
+    <t>2026-03-13T19:05:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -463,10 +463,10 @@
 </t>
   </si>
   <si>
-    <t>Unik identifikator(er) for episoden, som brukes ved rapportering til NPR</t>
-  </si>
-  <si>
-    <t>En eller flere unike identifikatorer (string og/eller UUID) som identifiserer episoden entydig i helseinstitusjonens systemer. Brukes ved rapportering til Norsk pasientregister (NPR). Kan inneholde både string-basert og UUID-basert identifikator samtidig.</t>
+    <t>NPR episodeidentifikator som sendes til LMDI</t>
+  </si>
+  <si>
+    <t>Unik identifikator for episoden som skal sendes til LMDI. Selv om helseinstitusjonens systemer kan ha flere NPR-identifiere for samme episode lokalt, skal kun én NPR-identifikator angis ved innsending til LMDI. Dersom flere identifiere finnes, velges gjerne den første eller foretrukne identifikatoren lokalt. Den valgte identifikatoren skal oppgis med sin string-representasjon og/eller UUID-representasjon dersom begge er tilgjengelig.</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1

</xml_diff>

<commit_message>
LMDI: Merge pull request #65 from folkehelseinstituttet/feat/update-npr-episode-identifier-definition
Oppdater definisjon av nprEpisodeIdentifier 474354a1cb9f13b9de99bd008abe2bc84ab3ba94
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-encounter.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-encounter.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-13T19:33:48+00:00</t>
+    <t>2026-03-13T19:51:56+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -466,7 +466,7 @@
     <t>NPR episodeidentifikator som sendes til LMDI</t>
   </si>
   <si>
-    <t>Unik identifikator for episoden som skal sendes til LMDI. Selv om helseinstitusjonens systemer kan ha flere NPR-identifiere for samme episode lokalt, skal kun én NPR-identifikator angis ved innsending til LMDI. Dersom flere identifiere finnes, velges gjerne den første eller foretrukne identifikatoren lokalt. Den valgte identifikatoren skal oppgis med sin string-representasjon og/eller UUID-representasjon dersom begge er tilgjengelig.</t>
+    <t>Unik identifikator for episoden som skal sendes til LMDI. Selv om avsender kan ha flere NPR-identifiere for samme episode lokalt, skal kun én NPR-identifikator angis ved innsending til LMDI. Dersom flere identifiere finnes, velges gjerne den første eller foretrukne identifikatoren lokalt. Den valgte identifikatoren skal oppgis med sin string-representasjon og/eller UUID-representasjon dersom begge er tilgjengelig.</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1

</xml_diff>

<commit_message>
LMDI: Merge pull request #76 from folkehelseinstituttet/fix/npr-episode-identifier-beskrivelser
Oppdater beskrivelser for nprEpisodeIdentifier 67b655153c2166ee16968e0b6f87611df7d3dbc2
</commit_message>
<xml_diff>
--- a/currentbuild/StructureDefinition-lmdi-encounter.xlsx
+++ b/currentbuild/StructureDefinition-lmdi-encounter.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-19T20:30:35+00:00</t>
+    <t>2026-03-20T06:49:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -463,10 +463,10 @@
 </t>
   </si>
   <si>
-    <t>NPR episodeidentifikator som sendes til LMDI</t>
-  </si>
-  <si>
-    <t>Unik identifikator for episoden som skal sendes til LMDI. Selv om avsender kan ha flere NPR-identifiere for samme episode lokalt, skal kun én NPR-identifikator angis ved innsending til LMDI. Dersom flere identifiere finnes, velges gjerne den første eller foretrukne identifikatoren lokalt. Den valgte identifikatoren skal oppgis med sin string-representasjon og/eller UUID-representasjon dersom begge er tilgjengelig.</t>
+    <t>Unik identifikator for episoden, som brukt i rapportering til Norsk pasientregister (NPR).</t>
+  </si>
+  <si>
+    <t>Unik identifikator for episoden, som brukt i rapportering til Norsk pasientregister (NPR). Hvis det er registrert flere NPR-identifiere for samme episode lokalt, skal kun én NPR-identifikator angis ved innsending til Legemiddelregisteret (LMR). Velg enten den første eller den lokalt foretrukne identifikatoren. Den valgte identifikatoren skal oppgis med sin string-representasjon og/eller UUID-representasjon, dersom begge er tilgjengelige oppgis begge.</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1

</xml_diff>